<commit_message>
AH SEO workbook: remove backlink outreach, .us launch, GA4/GSC access, and NAP/citation tasks per client direction
</commit_message>
<xml_diff>
--- a/decks/adriana-hoyos/seo-implementation-workbook.xlsx
+++ b/decks/adriana-hoyos/seo-implementation-workbook.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quote Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 - Foundation" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 - B2B Build" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded - Phase 3" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded - Out of Scope" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Targets" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Reference" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access &amp; Dependencies" sheetId="8" state="visible" r:id="rId8"/>
@@ -607,7 +607,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>7. Excluded / Phase 3 tab documents what was deliberately left out of this quote and why — do not price it in.</t>
+          <t>7. Excluded / Out of Scope tab documents what was deliberately left out of this quote and why — do not price it in.</t>
         </is>
       </c>
     </row>
@@ -696,15 +696,15 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTA('Phase 1 - Foundation'!A2:A9)</f>
+        <f>COUNTA('Phase 1 - Foundation'!A2:A8)</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>'Phase 1 - Foundation'!I10</f>
+        <f>'Phase 1 - Foundation'!I9</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Phase 1 - Foundation'!J10</f>
+        <f>'Phase 1 - Foundation'!J9</f>
         <v/>
       </c>
     </row>
@@ -715,15 +715,15 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTA('Phase 2 - B2B Build'!A2:A8)</f>
+        <f>COUNTA('Phase 2 - B2B Build'!A2:A5)</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>'Phase 2 - B2B Build'!I9</f>
+        <f>'Phase 2 - B2B Build'!I6</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>'Phase 2 - B2B Build'!J9</f>
+        <f>'Phase 2 - B2B Build'!J6</f>
         <v/>
       </c>
     </row>
@@ -749,7 +749,7 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Note: Phase 3 (franchisee playbook templating) is intentionally excluded from this quote — see 'Excluded - Phase 3' tab.</t>
+          <t>Note: Franchisee playbook templating, .us site work, local citation/NAP work, GA4/GSC access, and press backlink outreach are intentionally excluded from this quote — see 'Excluded - Out of Scope' tab.</t>
         </is>
       </c>
     </row>
@@ -763,478 +763,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>Page / Scope</t>
-        </is>
-      </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>Current State</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
-        <is>
-          <t>Target State</t>
-        </is>
-      </c>
-      <c r="F1" s="8" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="G1" s="8" t="inlineStr">
-        <is>
-          <t>Access Needed</t>
-        </is>
-      </c>
-      <c r="H1" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="I1" s="8" t="inlineStr">
-        <is>
-          <t>Est. Hours</t>
-        </is>
-      </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>Est. Cost</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>P1-01</t>
-        </is>
-      </c>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>Consolidate homepage H1 tags</t>
-        </is>
-      </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>Homepage</t>
-        </is>
-      </c>
-      <c r="D2" s="16" t="inlineStr">
-        <is>
-          <t>28 H1 tags found (confirmed via JS-rendered DOM audit)</t>
-        </is>
-      </c>
-      <c r="E2" s="16" t="inlineStr">
-        <is>
-          <t>Single canonical H1</t>
-        </is>
-      </c>
-      <c r="F2" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G2" s="16" t="inlineStr">
-        <is>
-          <t>CMS/dev</t>
-        </is>
-      </c>
-      <c r="H2" s="16" t="inlineStr">
-        <is>
-          <t>Confirm which templating component is injecting duplicate H1s before removing</t>
-        </is>
-      </c>
-      <c r="I2" s="17" t="n"/>
-      <c r="J2" s="18">
-        <f>IF(I2="","",I2*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>P1-02</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Implement structured data / schema markup</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Sitewide (homepage, locations, product pages)</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>No LocalBusiness, Organization, or Product schema found on any page reviewed</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>Schema deployed sitewide</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G3" s="16" t="inlineStr">
-        <is>
-          <t>CMS/dev</t>
-        </is>
-      </c>
-      <c r="H3" s="16" t="inlineStr">
-        <is>
-          <t>Prerequisite for local-pack visibility once city pages launch in Phase 2</t>
-        </is>
-      </c>
-      <c r="I3" s="17" t="n"/>
-      <c r="J3" s="18">
-        <f>IF(I3="","",I3*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>P1-03</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Write custom meta descriptions</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Homepage, /locations/, product category pages</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>Missing — Google auto-generates snippet text</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Custom, keyword-aligned meta descriptions</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="inlineStr">
-        <is>
-          <t>CMS/dev + copywriting</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>Coordinate voice/tone with brand team (Constanza)</t>
-        </is>
-      </c>
-      <c r="I4" s="17" t="n"/>
-      <c r="J4" s="18">
-        <f>IF(I4="","",I4*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>P1-04</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Resolve keyword cannibalization — "Design Studio" cluster</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>20+ pages</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>20+ pages competing for "adriana hoyos design studio," positions 2–75</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>One canonical page; others redirected or canonicalized</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr">
-        <is>
-          <t>CMS/dev + IA decision</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="inlineStr">
-        <is>
-          <t>Ties to the confirmed decision to keep the Design Studio subdomain separate</t>
-        </is>
-      </c>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="18">
-        <f>IF(I5="","",I5*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>P1-05</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Resolve keyword cannibalization — dining chairs cluster</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>47 URLs</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>"adriana hoyos dining chairs" competes across 47 separate URLs</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Canonical product/category page identified and reinforced</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>CMS/dev</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="18">
-        <f>IF(I6="","",I6*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>P1-06</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Noindex the Design Studio subdomain</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>adrianahoyosdesignstudio.com</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Indexable, competing with furnishing-business keywords</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>robots.txt noindex directive applied</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
-        <is>
-          <t>Subdomain hosting/DNS access</t>
-        </is>
-      </c>
-      <c r="H7" s="16" t="inlineStr">
-        <is>
-          <t>Client confirmed on 7/10/26 call this should stay separate and unindexed</t>
-        </is>
-      </c>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="18">
-        <f>IF(I7="","",I7*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>P1-07</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Press backlink dofollow outreach</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Architectural Digest (2 links), Robb Report (1 link)</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Both nofollow — no authority passed</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>Dofollow requested on next placements with each publication</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>PR/comms relationship (not technical)</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>Elle Decor's existing link is already dofollow (Page AS 34) — no action needed there</t>
-        </is>
-      </c>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="18">
-        <f>IF(I8="","",I8*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>P1-08</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Referring-domain decline investigation</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Sitewide backlink profile</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Referring domains down from ~900 (year prior) to 657 (May '26) to 578 (Jul '26)</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Root causes identified; priority reclamation list built</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Backlink Analytics (in hand) + outreach capacity</t>
-        </is>
-      </c>
-      <c r="H9" s="16" t="inlineStr">
-        <is>
-          <t>Trend is still declining as of this pull</t>
-        </is>
-      </c>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="18">
-        <f>IF(I9="","",I9*'Quote Summary'!$B$3)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="n"/>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>Phase 1 Subtotal</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="13">
-        <f>SUM(I2:I9)</f>
-        <v/>
-      </c>
-      <c r="J10" s="14">
-        <f>SUM(J2:J9)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1310,27 +838,27 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>P2-01</t>
+          <t>P1-01</t>
         </is>
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>Build Trade Program / Become a Franchisee hub</t>
+          <t>Consolidate homepage H1 tags</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>New page(s) on .com</t>
+          <t>Homepage</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>Does not exist</t>
+          <t>28 H1 tags found (confirmed via JS-rendered DOM audit)</t>
         </is>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>Staged page with context before any login wall (model: Caracole, Bernhardt)</t>
+          <t>Single canonical H1</t>
         </is>
       </c>
       <c r="F2" s="16" t="inlineStr">
@@ -1340,12 +868,12 @@
       </c>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t>GA/GSC access + content + dev</t>
+          <t>CMS/dev</t>
         </is>
       </c>
       <c r="H2" s="16" t="inlineStr">
         <is>
-          <t>Primary landing page for the entire 'trade program' keyword cluster</t>
+          <t>Confirm which templating component is injecting duplicate H1s before removing</t>
         </is>
       </c>
       <c r="I2" s="17" t="n"/>
@@ -1357,27 +885,27 @@
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>P2-02</t>
+          <t>P1-02</t>
         </is>
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Launch .us with city-based URL structure</t>
+          <t>Implement structured data / schema markup</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>New domain: .us</t>
+          <t>Sitewide (homepage, locations, product pages)</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Not live</t>
+          <t>No LocalBusiness, Organization, or Product schema found on any page reviewed</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>Live with subfolder structure (/us/dc, /us/austin, /us/coral-gables)</t>
+          <t>Schema deployed sitewide</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -1387,12 +915,12 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>DNS/hosting + dev</t>
+          <t>CMS/dev</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Coordinate URL structure with Meta ad-account naming (marketing team)</t>
+          <t>Prerequisite for local-pack visibility once city pages launch in Phase 2</t>
         </is>
       </c>
       <c r="I3" s="17" t="n"/>
@@ -1404,42 +932,42 @@
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>P2-03</t>
+          <t>P1-03</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Build individual location pages</t>
+          <t>Write custom meta descriptions</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Coral Gables, DC (initial 2 cities)</t>
+          <t>Homepage, /locations/, product category pages</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Single shared /locations/ page — 1 visit/month</t>
+          <t>Missing — Google auto-generates snippet text</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>Dedicated page per city, each with local schema</t>
+          <t>Custom, keyword-aligned meta descriptions</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>Dev + content</t>
+          <t>CMS/dev + copywriting</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>Template this build so it's replicable for future cities</t>
+          <t>Coordinate voice/tone with brand team (Constanza)</t>
         </is>
       </c>
       <c r="I4" s="17" t="n"/>
@@ -1451,42 +979,42 @@
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>P2-04</t>
+          <t>P1-04</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Trade-program content build</t>
+          <t>Resolve keyword cannibalization — "Design Studio" cluster</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Trade Program hub + supporting pages</t>
+          <t>20+ pages</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>Zero ranking keywords in this cluster</t>
+          <t>20+ pages competing for "adriana hoyos design studio," positions 2–75</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Target "interior design trade programs," "interior designer trade program," "trade programs for interior designers"</t>
+          <t>One canonical page; others redirected or canonicalized</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Content writer + SEO</t>
+          <t>CMS/dev + IA decision</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>See Keyword Targets tab for full cluster and volumes</t>
+          <t>Ties to the confirmed decision to keep the Design Studio subdomain separate</t>
         </is>
       </c>
       <c r="I5" s="17" t="n"/>
@@ -1498,44 +1026,40 @@
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>P2-05</t>
+          <t>P1-05</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Franchise-opportunity content build</t>
+          <t>Resolve keyword cannibalization — dining chairs cluster</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Franchise hub page</t>
+          <t>47 URLs</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Zero ranking keywords in this cluster</t>
+          <t>"adriana hoyos dining chairs" competes across 47 separate URLs</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Target "furniture franchise opportunities," "furniture franchise"</t>
+          <t>Canonical product/category page identified and reinforced</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Content writer + SEO</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>Low volume (70/mo top term) but currently uncontested past BoConcept's #3</t>
-        </is>
-      </c>
+          <t>CMS/dev</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr"/>
       <c r="I6" s="17" t="n"/>
       <c r="J6" s="18">
         <f>IF(I6="","",I6*'Quote Summary'!$B$3)</f>
@@ -1545,42 +1069,42 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>P2-06</t>
+          <t>P1-06</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Secure GA4 / GSC access and run full baseline audit</t>
+          <t>Noindex the Design Studio subdomain</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Client analytics accounts</t>
+          <t>adrianahoyosdesignstudio.com</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Not yet granted</t>
+          <t>Indexable, competing with furnishing-business keywords</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>Full keyword/traffic baseline established for precise Phase 2 scoping</t>
+          <t>robots.txt noindex directive applied</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
-          <t>Critical — blocks precise scoping</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Client IT / Alegria</t>
+          <t>Subdomain hosting/DNS access</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Requested on the 7/10/26 call; still pending as of this workbook</t>
+          <t>Client confirmed on 7/10/26 call this should stay separate and unindexed</t>
         </is>
       </c>
       <c r="I7" s="17" t="n"/>
@@ -1592,40 +1116,44 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>P2-07</t>
+          <t>P1-07</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Local citation / NAP consistency pass</t>
+          <t>Referring-domain decline investigation</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Coral Gables + DC (and future cities)</t>
+          <t>Sitewide backlink profile</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Unverified across directories and Google Business Profile</t>
+          <t>Referring domains down from ~900 (year prior) to 657 (May '26) to 578 (Jul '26)</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Consistent NAP sitewide and across major directories</t>
+          <t>Root causes identified; priority reclamation list built</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Google Business Profile admin access</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr"/>
+          <t>Backlink Analytics (in hand) + outreach capacity</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Trend is still declining as of this pull</t>
+        </is>
+      </c>
       <c r="I8" s="17" t="n"/>
       <c r="J8" s="18">
         <f>IF(I8="","",I8*'Quote Summary'!$B$3)</f>
@@ -1636,7 +1164,7 @@
       <c r="A9" s="19" t="n"/>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Phase 2 Subtotal</t>
+          <t>Phase 1 Subtotal</t>
         </is>
       </c>
       <c r="C9" s="19" t="n"/>
@@ -1651,6 +1179,294 @@
       </c>
       <c r="J9" s="14">
         <f>SUM(J2:J8)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Page / Scope</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Current State</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Target State</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Access Needed</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Est. Hours</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Est. Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>P2-01</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Build Trade Program / Become a Franchisee hub</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>New page(s) on .com</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Does not exist</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>Staged page with context before any login wall (model: Caracole, Bernhardt)</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>GA/GSC access + content + dev</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
+        <is>
+          <t>Primary landing page for the entire 'trade program' keyword cluster</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="18">
+        <f>IF(I2="","",I2*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>P2-02</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Build individual location pages</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Coral Gables, DC (initial 2 cities)</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Single shared /locations/ page — 1 visit/month</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Dedicated page per city, each with local schema</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Dev + content</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Template this build so it's replicable for future cities</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="18">
+        <f>IF(I3="","",I3*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Trade-program content build</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Trade Program hub + supporting pages</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Zero ranking keywords in this cluster</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Target "interior design trade programs," "interior designer trade program," "trade programs for interior designers"</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>Content writer + SEO</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>See Keyword Targets tab for full cluster and volumes</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="18">
+        <f>IF(I4="","",I4*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Franchise-opportunity content build</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Franchise hub page</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Zero ranking keywords in this cluster</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Target "furniture franchise opportunities," "furniture franchise"</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Content writer + SEO</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Low volume (70/mo top term) but currently uncontested past BoConcept's #3</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="18">
+        <f>IF(I5="","",I5*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Phase 2 Subtotal</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="19" t="n"/>
+      <c r="I6" s="13">
+        <f>SUM(I2:I5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="14">
+        <f>SUM(J2:J5)</f>
         <v/>
       </c>
     </row>
@@ -1665,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1715,6 +1531,94 @@
       <c r="D2" s="16" t="inlineStr">
         <is>
           <t>Once the DC location is live and a second franchisee city is identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>.us domain launch</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Launch .us with city-based subfolder structure (/us/dc, /us/austin, /us/coral-gables) for localized campaign infrastructure.</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Client direction, Jul 2026: no work on the .us site in this scope.</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>If client direction changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Local citation / NAP consistency pass</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Audit and align Name/Address/Phone consistency across Google Business Profile and directories for Coral Gables and DC.</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Client direction, Jul 2026: no local SEO / citation work in this scope.</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>If client direction changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Secure GA4 / GSC access and baseline audit</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Get client analytics access granted and run a full keyword/traffic baseline to sharpen Phase 2 scoping.</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Removed per client direction, Jul 2026.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>If client direction changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Press backlink dofollow outreach</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Request dofollow status on future Architectural Digest and Robb Report placements.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Removed per client direction, Jul 2026.</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>If client direction changes</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2622,154 +2526,66 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Google Analytics 4 access</t>
+          <t>Semrush API units</t>
         </is>
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>Not yet granted</t>
+          <t>Exhausted on EmberTribe account as of Jul '26</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>Precise Phase 2 keyword/traffic targeting</t>
+          <t>Refreshed live competitive tracking</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>Alegria (client)</t>
+          <t>EmberTribe internal</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
-          <t>Google Search Console access</t>
+          <t>CMS / dev platform access</t>
         </is>
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Not yet granted</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>Precise Phase 2 keyword/traffic targeting</t>
+          <t>All Phase 1 technical fixes</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Alegria (client)</t>
+          <t>Christopher (client)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Semrush API units</t>
+          <t>Design Studio subdomain hosting access</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Exhausted on EmberTribe account as of Jul '26</t>
+          <t>Status unknown</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Refreshed live competitive tracking</t>
+          <t>robots.txt noindex task (P1-06)</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>EmberTribe internal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>CMS / dev platform access</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Not yet confirmed</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>All Phase 1 technical fixes</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
           <t>Christopher (client)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>.us domain registration / DNS</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Status unknown</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Phase 2 launch</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Alegria / Christopher (client)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Design Studio subdomain hosting access</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Status unknown</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>robots.txt noindex task (P1-06)</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Christopher (client)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Google Business Profile admin access</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Status unknown</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>Local citation/NAP work (P2-07)</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Alegria (client)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AH SEO workbook: replace Design Studio/dining chairs cannibalization tasks with verified findings (hreflang duplicate-content fix, PDF noindex, Design Studio page decision)
</commit_message>
<xml_diff>
--- a/decks/adriana-hoyos/seo-implementation-workbook.xlsx
+++ b/decks/adriana-hoyos/seo-implementation-workbook.xlsx
@@ -696,15 +696,15 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTA('Phase 1 - Foundation'!A2:A8)</f>
+        <f>COUNTA('Phase 1 - Foundation'!A2:A9)</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>'Phase 1 - Foundation'!I9</f>
+        <f>'Phase 1 - Foundation'!I10</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'Phase 1 - Foundation'!J9</f>
+        <f>'Phase 1 - Foundation'!J10</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -984,37 +984,37 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Resolve keyword cannibalization — "Design Studio" cluster</t>
+          <t>Design Studio page-strategy decision</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>20+ pages</t>
+          <t>Main domain (about-us, blog, press pages)</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>20+ pages competing for "adriana hoyos design studio," positions 2–75</t>
+          <t>No dedicated Design Studio page exists on adrianahoyos.com — the term only appears incidentally in About Us copy, blog posts, and press releases (confirmed via Google index check, Jul 2026)</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>One canonical page; others redirected or canonicalized</t>
+          <t>Decision: build a dedicated page, or accept the term resolves to the (separate, noindexed) Design Studio subdomain</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>CMS/dev + IA decision</t>
+          <t>Strategy decision + CMS/dev if building</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Ties to the confirmed decision to keep the Design Studio subdomain separate</t>
+          <t>Not a redirect/consolidation task — there's no existing page to consolidate around. Originally described as '20+ competing pages'; real cause is incidental mentions, not competing landing pages</t>
         </is>
       </c>
       <c r="I5" s="17" t="n"/>
@@ -1031,27 +1031,27 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Resolve keyword cannibalization — dining chairs cluster</t>
+          <t>Implement hreflang / canonicalization — worldwide vs. /ec/ catalog</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>47 URLs</t>
+          <t>Entire product catalog (buffets, tables, chairs, etc.), not just dining chairs</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>"adriana hoyos dining chairs" competes across 47 separate URLs</t>
+          <t>/our-products/dining-room/chairs/ and /ec/our-products/dining-room/chairs/ are near-duplicate pages competing in Google's index — confirmed the /ec/ path mirrors the full catalog, not one product line</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Canonical product/category page identified and reinforced</t>
+          <t>hreflang tags (or canonical tags if no genuine regional content difference) implemented sitewide between worldwide and /ec/ paths</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
@@ -1059,7 +1059,11 @@
           <t>CMS/dev</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr"/>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Originally described as '47 competing URLs for dining chairs'; real cause is a sitewide international-duplicate-content pattern</t>
+        </is>
+      </c>
       <c r="I6" s="17" t="n"/>
       <c r="J6" s="18">
         <f>IF(I6="","",I6*'Quote Summary'!$B$3)</f>
@@ -1074,22 +1078,22 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Noindex the Design Studio subdomain</t>
+          <t>Noindex PDF spec sheets competing in search</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>adrianahoyosdesignstudio.com</t>
+          <t>wp-content/uploads product spec PDFs (e.g. RM01-400.pdf, GM02-142.pdf, BR01-210.pdf)</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>Indexable, competing with furnishing-business keywords</t>
+          <t>Indexed PDF spec sheets compete with product/category pages for the same terms</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>robots.txt noindex directive applied</t>
+          <t>noindex via X-Robots-Tag header on the PDF directory, or move behind a non-crawlable path</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -1099,12 +1103,12 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Subdomain hosting/DNS access</t>
+          <t>CMS/dev or server config access</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>Client confirmed on 7/10/26 call this should stay separate and unindexed</t>
+          <t>Discovered via Google index check, Jul 2026 — part of the same cannibalization pattern as P1-05</t>
         </is>
       </c>
       <c r="I7" s="17" t="n"/>
@@ -1121,22 +1125,22 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Referring-domain decline investigation</t>
+          <t>Noindex the Design Studio subdomain</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>Sitewide backlink profile</t>
+          <t>adrianahoyosdesignstudio.com</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>Referring domains down from ~900 (year prior) to 657 (May '26) to 578 (Jul '26)</t>
+          <t>Indexable, competing with furnishing-business keywords</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Root causes identified; priority reclamation list built</t>
+          <t>robots.txt noindex directive applied</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
@@ -1146,12 +1150,12 @@
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Backlink Analytics (in hand) + outreach capacity</t>
+          <t>Subdomain hosting/DNS access</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>Trend is still declining as of this pull</t>
+          <t>Client confirmed on 7/10/26 call this should stay separate and unindexed</t>
         </is>
       </c>
       <c r="I8" s="17" t="n"/>
@@ -1161,24 +1165,71 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n"/>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>P1-08</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Referring-domain decline investigation</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Sitewide backlink profile</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Referring domains down from ~900 (year prior) to 657 (May '26) to 578 (Jul '26)</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Root causes identified; priority reclamation list built</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Backlink Analytics (in hand) + outreach capacity</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Trend is still declining as of this pull</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="18">
+        <f>IF(I9="","",I9*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Phase 1 Subtotal</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="19" t="n"/>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="13">
-        <f>SUM(I2:I8)</f>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="13">
+        <f>SUM(I2:I9)</f>
         <v/>
       </c>
-      <c r="J9" s="14">
-        <f>SUM(J2:J8)</f>
+      <c r="J10" s="14">
+        <f>SUM(J2:J9)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
AH SEO workbook: split Trade Program hub and Become a Franchisee hub into two distinct Phase 2 tasks
</commit_message>
<xml_diff>
--- a/decks/adriana-hoyos/seo-implementation-workbook.xlsx
+++ b/decks/adriana-hoyos/seo-implementation-workbook.xlsx
@@ -715,15 +715,15 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTA('Phase 2 - B2B Build'!A2:A5)</f>
+        <f>COUNTA('Phase 2 - B2B Build'!A2:A6)</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>'Phase 2 - B2B Build'!I6</f>
+        <f>'Phase 2 - B2B Build'!I7</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>'Phase 2 - B2B Build'!J6</f>
+        <f>'Phase 2 - B2B Build'!J7</f>
         <v/>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B2" s="16" t="inlineStr">
         <is>
-          <t>Build Trade Program / Become a Franchisee hub</t>
+          <t>Build Trade Program hub</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>New page(s) on .com</t>
+          <t>New page on .com</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>Staged page with context before any login wall (model: Caracole, Bernhardt)</t>
+          <t>Staged page with context before any login wall (model: Caracole, Bernhardt), for interior designers and dealers</t>
         </is>
       </c>
       <c r="F2" s="16" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H2" s="16" t="inlineStr">
         <is>
-          <t>Primary landing page for the entire 'trade program' keyword cluster</t>
+          <t>Primary landing page for the entire 'trade program' keyword cluster. Split out from franchise hub — different audience, different content (pricing/account access vs. investment figures)</t>
         </is>
       </c>
       <c r="I2" s="17" t="n"/>
@@ -1366,22 +1366,22 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Build individual location pages</t>
+          <t>Build Become a Franchisee hub</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
         <is>
-          <t>Coral Gables, DC (initial 2 cities)</t>
+          <t>New page on .com</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Single shared /locations/ page — 1 visit/month</t>
+          <t>Does not exist</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>Dedicated page per city, each with local schema</t>
+          <t>Dedicated franchise page for prospective franchisees (model: BoConcept) — territory/criteria and path to inquire</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -1391,12 +1391,12 @@
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Dev + content</t>
+          <t>Content + dev + client input on what can be disclosed (investment figures, territory criteria)</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Template this build so it's replicable for future cities</t>
+          <t>Primary landing page for the 'franchise opportunities' keyword cluster. Split out from trade program hub</t>
         </is>
       </c>
       <c r="I3" s="17" t="n"/>
@@ -1413,37 +1413,37 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Trade-program content build</t>
+          <t>Build individual location pages</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Trade Program hub + supporting pages</t>
+          <t>Coral Gables, DC (initial 2 cities)</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Zero ranking keywords in this cluster</t>
+          <t>Single shared /locations/ page — 1 visit/month</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>Target "interior design trade programs," "interior designer trade program," "trade programs for interior designers"</t>
+          <t>Dedicated page per city, each with local schema</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>Content writer + SEO</t>
+          <t>Dev + content</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>See Keyword Targets tab for full cluster and volumes</t>
+          <t>Template this build so it's replicable for future cities</t>
         </is>
       </c>
       <c r="I4" s="17" t="n"/>
@@ -1460,12 +1460,12 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Franchise-opportunity content build</t>
+          <t>Trade-program content build</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Franchise hub page</t>
+          <t>Trade Program hub + supporting pages</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>Target "furniture franchise opportunities," "furniture franchise"</t>
+          <t>Target "interior design trade programs," "interior designer trade program," "trade programs for interior designers"</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Low volume (70/mo top term) but currently uncontested past BoConcept's #3</t>
+          <t>See Keyword Targets tab for full cluster and volumes</t>
         </is>
       </c>
       <c r="I5" s="17" t="n"/>
@@ -1500,24 +1500,71 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n"/>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>P2-05</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Franchise-opportunity content build</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Franchise hub page</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Zero ranking keywords in this cluster</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>Target "furniture franchise opportunities," "furniture franchise"</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>Content writer + SEO</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Low volume (70/mo top term) but currently uncontested past BoConcept's #3</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="18">
+        <f>IF(I6="","",I6*'Quote Summary'!$B$3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Phase 2 Subtotal</t>
         </is>
       </c>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="13">
-        <f>SUM(I2:I5)</f>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="13">
+        <f>SUM(I2:I6)</f>
         <v/>
       </c>
-      <c r="J6" s="14">
-        <f>SUM(J2:J5)</f>
+      <c r="J7" s="14">
+        <f>SUM(J2:J6)</f>
         <v/>
       </c>
     </row>

</xml_diff>